<commit_message>
hashing utils for path as PK created
</commit_message>
<xml_diff>
--- a/docs/en/CollisionProbability.xlsx
+++ b/docs/en/CollisionProbability.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repos\jpjsm@github\simplify\docs\en\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9EF178A3-0545-4794-8299-5A0E7F181B76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8E21DCD-A411-4B76-BE5D-A716C5175B3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ECA767C8-6D9E-4745-946A-6BC4E68755CA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="Hash_Size_bits">Sheet1!$E$1</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>n</t>
   </si>
@@ -58,6 +61,9 @@
   <si>
     <t>Probability</t>
   </si>
+  <si>
+    <t>Hash Size (bits)</t>
+  </si>
 </sst>
 </file>
 
@@ -65,9 +71,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="167" formatCode="0.000%"/>
-    <numFmt numFmtId="171" formatCode="_(* #,##0.000000_);_(* \(#,##0.000000\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="0.000%"/>
+    <numFmt numFmtId="166" formatCode="_(* #,##0.000000_);_(* \(#,##0.000000\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -122,18 +128,18 @@
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="171" fontId="2" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="2" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Accent4" xfId="3" builtinId="41"/>
@@ -471,7 +477,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B5E1603-4B10-4703-AE4F-6078242F27AF}">
-  <dimension ref="B1:H8"/>
+  <dimension ref="B1:H10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="15.28515625" style="1" bestFit="1" customWidth="1"/>
@@ -483,226 +489,234 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="C1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="C3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2">
-        <v>4</v>
-      </c>
-      <c r="C2" s="1">
-        <f>POWER(10,B2)</f>
-        <v>10000</v>
-      </c>
-      <c r="D2" s="2">
-        <f>C2*C2</f>
-        <v>100000000</v>
-      </c>
-      <c r="E2">
-        <f>-(D2/POWER(2,65))</f>
-        <v>-2.7105054312137611E-12</v>
-      </c>
-      <c r="F2" s="6">
-        <f>EXP(E2)</f>
-        <v>0.9999999999972895</v>
-      </c>
-      <c r="G2">
-        <f>1-F2</f>
-        <v>2.7104984923198572E-12</v>
-      </c>
-      <c r="H2" s="4">
-        <f>G2</f>
-        <v>2.7104984923198572E-12</v>
-      </c>
-    </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B3">
-        <v>5</v>
-      </c>
-      <c r="C3" s="1">
-        <f t="shared" ref="C3:C8" si="0">POWER(10,B3)</f>
-        <v>100000</v>
-      </c>
-      <c r="D3" s="2">
-        <f t="shared" ref="D3:D8" si="1">C3*C3</f>
-        <v>10000000000</v>
-      </c>
-      <c r="E3">
-        <f t="shared" ref="E3:E8" si="2">-(D3/POWER(2,65))</f>
-        <v>-2.7105054312137611E-10</v>
-      </c>
-      <c r="F3" s="6">
-        <f t="shared" ref="F3:F8" si="3">EXP(E3)</f>
-        <v>0.99999999972894948</v>
-      </c>
-      <c r="G3">
-        <f t="shared" ref="G3:G8" si="4">1-F3</f>
-        <v>2.7105051536580049E-10</v>
-      </c>
-      <c r="H3" s="4">
-        <f t="shared" ref="H3:H8" si="5">G3</f>
-        <v>2.7105051536580049E-10</v>
       </c>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B4">
+        <v>4</v>
+      </c>
+      <c r="C4" s="1">
+        <f>POWER(10,B4)</f>
+        <v>10000</v>
+      </c>
+      <c r="D4" s="2">
+        <f>C4*(C4-1)</f>
+        <v>99990000</v>
+      </c>
+      <c r="E4">
+        <f>-(D4/POWER(2,Hash_Size_bits+1))</f>
+        <v>-6.3102561530439176E-22</v>
+      </c>
+      <c r="F4" s="6">
+        <f>EXP(E4)</f>
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <f>1-F4</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="4">
+        <f>G4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5" s="1">
+        <f t="shared" ref="C5:C10" si="0">POWER(10,B5)</f>
+        <v>100000</v>
+      </c>
+      <c r="D5" s="2">
+        <f t="shared" ref="D5:D10" si="1">C5*(C5-1)</f>
+        <v>9999900000</v>
+      </c>
+      <c r="E5">
+        <f>-(D5/POWER(2,Hash_Size_bits+1))</f>
+        <v>-6.3108241328956768E-20</v>
+      </c>
+      <c r="F5" s="6">
+        <f t="shared" ref="F5:F10" si="2">EXP(E5)</f>
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <f t="shared" ref="G5:G10" si="3">1-F5</f>
+        <v>0</v>
+      </c>
+      <c r="H5" s="4">
+        <f t="shared" ref="H5:H10" si="4">G5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B6">
         <v>6</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C6" s="1">
         <f t="shared" si="0"/>
         <v>1000000</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D6" s="2">
         <f t="shared" si="1"/>
-        <v>1000000000000</v>
-      </c>
-      <c r="E4">
+        <v>999999000000</v>
+      </c>
+      <c r="E6">
+        <f>-(D6/POWER(2,Hash_Size_bits+1))</f>
+        <v>-6.3108809308808527E-18</v>
+      </c>
+      <c r="F6" s="6">
         <f t="shared" si="2"/>
-        <v>-2.7105054312137611E-8</v>
-      </c>
-      <c r="F4" s="6">
+        <v>1</v>
+      </c>
+      <c r="G6">
         <f t="shared" si="3"/>
-        <v>0.99999997289494602</v>
-      </c>
-      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4">
         <f t="shared" si="4"/>
-        <v>2.7105053979070703E-8</v>
-      </c>
-      <c r="H4" s="4">
-        <f t="shared" si="5"/>
-        <v>2.7105053979070703E-8</v>
-      </c>
-    </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B7">
         <v>7</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C7" s="1">
         <f t="shared" si="0"/>
         <v>10000000</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D7" s="2">
         <f t="shared" si="1"/>
-        <v>100000000000000</v>
-      </c>
-      <c r="E5">
+        <v>99999990000000</v>
+      </c>
+      <c r="E7">
+        <f>-(D7/POWER(2,Hash_Size_bits+1))</f>
+        <v>-6.3108866106793703E-16</v>
+      </c>
+      <c r="F7" s="6">
         <f t="shared" si="2"/>
-        <v>-2.7105054312137611E-6</v>
-      </c>
-      <c r="F5" s="6">
+        <v>0.99999999999999933</v>
+      </c>
+      <c r="G7">
         <f t="shared" si="3"/>
-        <v>0.99999728949824218</v>
-      </c>
-      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H7" s="4">
         <f t="shared" si="4"/>
-        <v>2.7105017578188395E-6</v>
-      </c>
-      <c r="H5" s="4">
-        <f t="shared" si="5"/>
-        <v>2.7105017578188395E-6</v>
-      </c>
-    </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B8">
         <v>8</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C8" s="1">
         <f t="shared" si="0"/>
         <v>100000000</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D8" s="2">
         <f t="shared" si="1"/>
-        <v>1E+16</v>
-      </c>
-      <c r="E6">
+        <v>9999999900000000</v>
+      </c>
+      <c r="E8">
+        <f>-(D8/POWER(2,Hash_Size_bits+1))</f>
+        <v>-6.310887178659222E-14</v>
+      </c>
+      <c r="F8" s="6">
         <f t="shared" si="2"/>
-        <v>-2.7105054312137611E-4</v>
-      </c>
-      <c r="F6" s="6">
+        <v>0.99999999999993694</v>
+      </c>
+      <c r="G8">
         <f t="shared" si="3"/>
-        <v>0.99972898618775841</v>
-      </c>
-      <c r="G6">
+        <v>6.3060667798708891E-14</v>
+      </c>
+      <c r="H8" s="4">
         <f t="shared" si="4"/>
-        <v>2.7101381224159393E-4</v>
-      </c>
-      <c r="H6" s="4">
-        <f t="shared" si="5"/>
-        <v>2.7101381224159393E-4</v>
-      </c>
-    </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B7">
+        <v>6.3060667798708891E-14</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B9">
         <v>9</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C9" s="1">
         <f t="shared" si="0"/>
         <v>1000000000</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D9" s="2">
         <f t="shared" si="1"/>
-        <v>1E+18</v>
-      </c>
-      <c r="E7">
+        <v>9.99999999E+17</v>
+      </c>
+      <c r="E9">
+        <f>-(D9/POWER(2,Hash_Size_bits+1))</f>
+        <v>-6.3108872354572072E-12</v>
+      </c>
+      <c r="F9" s="6">
         <f t="shared" si="2"/>
-        <v>-2.7105054312137611E-2</v>
-      </c>
-      <c r="F7" s="6">
+        <v>0.99999999999368916</v>
+      </c>
+      <c r="G9">
         <f t="shared" si="3"/>
-        <v>0.97325899109966507</v>
-      </c>
-      <c r="G7">
+        <v>6.3108407388767773E-12</v>
+      </c>
+      <c r="H9" s="4">
         <f t="shared" si="4"/>
-        <v>2.6741008900334928E-2</v>
-      </c>
-      <c r="H7" s="4">
-        <f t="shared" si="5"/>
-        <v>2.6741008900334928E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B8">
+        <v>6.3108407388767773E-12</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B10">
         <v>10</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C10" s="1">
         <f t="shared" si="0"/>
         <v>10000000000</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D10" s="2">
         <f t="shared" si="1"/>
-        <v>1E+20</v>
-      </c>
-      <c r="E8">
+        <v>9.9999999989999993E+19</v>
+      </c>
+      <c r="E10">
+        <f>-(D10/POWER(2,Hash_Size_bits+1))</f>
+        <v>-6.3108872411370053E-10</v>
+      </c>
+      <c r="F10" s="6">
         <f t="shared" si="2"/>
-        <v>-2.7105054312137611</v>
-      </c>
-      <c r="F8" s="6">
+        <v>0.99999999936891126</v>
+      </c>
+      <c r="G10">
         <f t="shared" si="3"/>
-        <v>6.6503185433377424E-2</v>
-      </c>
-      <c r="G8">
+        <v>6.3108873682438116E-10</v>
+      </c>
+      <c r="H10" s="4">
         <f t="shared" si="4"/>
-        <v>0.93349681456662259</v>
-      </c>
-      <c r="H8" s="4">
-        <f t="shared" si="5"/>
-        <v>0.93349681456662259</v>
+        <v>6.3108873682438116E-10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>